<commit_message>
Add SPARQL-vs-SQL comparison, ontology viz, scoring, and CQ15
- bgg_agents_slides.pptx: 24-slide presentation; added QSQL1-8 comparison
  section, QSQL4/QSQL8 deep-dive slides, slide 3 run instructions
- bgg_sparql_compare.py / bgg_sql_compare.py: added QSQL3-8, generated_query
  logging to qa_log.jsonl
- bgg_sparql_qa.ipynb: fixed SYSTEM_SPARQL stored char-by-char (337 lines now)
- GoldenQandA_June17.*: added CQ15 (expansion counts) to all three formats
- qa_log.jsonl: all entries auto-scored via Claude Haiku (_autoscore.py)
- report.xlsx: updated with QSQL8 row and CQ15 scores
- bgg_ontology_diagram.png: static class/edge diagram (matplotlib)
- bgg_ontology_interactive.html: interactive vis.js graph with expandable nodes
- Helper scripts: _add_qsql8.py, _add_qsql4_slide.py, _fill_slide3.py,
  _autoscore.py, _viz_ontology.py, _gen_ontology_html.py

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SQL vs SPARQL" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Agent Comparison" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="QA Scores" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Key Observations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL vs SPARQL" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Comparison" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Scores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Observations" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -53,7 +53,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -125,6 +125,16 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -180,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -246,6 +256,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -611,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -958,29 +971,77 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>QSQL8</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Total reimplementation family size (any depth, no anchor)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>861 games returned; top: CATAN 33, Love Letter 25, TtR 21</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>bgg:reimplements+ counts full descendant tree in one token; identical structure to depth-1 query plus one character</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>861 games returned; identical results</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>10</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>WITH RECURSIVE needed to compute transitive closure before GROUP BY; requires full query restructure vs SPARQL's single + token</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>KEY INSIGHT</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="80" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>QSQL6 (community detection) is the clearest demonstration: SPARQL expresses arbitrary-depth transitive graph traversal in a single property-path line ((bgg:hasOwnershipOf/^bgg:hasOwnershipOf)+) while SQL requires a 15-line WITH RECURSIVE CTE. Furthermore the SQL LLM introduced a subtle correctness bug — Susanne herself was re-added to her own community via the recursive arm — yielding 203 instead of the correct 202. SPARQL's FILTER naturally avoided this.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="50" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
-        <is>
-          <t>QSQL7 also shows SPARQL's advantage: bgg:reimplements* traverses the entire Ticket to Ride reimplementation family (any depth) in one expression, vs an 8-line recursive CTE in SQL. Both return 22 games correctly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="22" t="inlineStr">
+    <row r="13" ht="50" customHeight="1"/>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>QSQL7 also shows SPARQL's advantage: bgg:reimplements* traverses the entire Ticket to Ride reimplementation family (any depth) in one expression, vs an 8-line recursive CTE in SQL. Both return 22 games correctly.
+QSQL8 (anchorless family size) is the clearest one-token demonstration: adding + to bgg:reimplements gives full transitive family counts across all 861 games in the database. SQL needs a WITH RECURSIVE CTE to do the same. Both return identical results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1"/>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>WITH RECURSIVE adoption note: Although supported by all major SQL engines (PostgreSQL, SQLite, MySQL 8+, SQL Server), WITH RECURSIVE is rarely used in practice. Most developers avoid it, resorting to application-level traversal, depth-limited self-joins, or denormalized closure tables. SPARQL property paths (+, *, ^) are the standard idiom — every SPARQL user knows them.</t>
         </is>
@@ -1002,7 +1063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1332,6 +1393,33 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Cost per 20-question run</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>~$0.30</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>~$0.04</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>~$0.80</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>~$3.00 (paid) / ~$0 (free tier)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1343,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1421,7 +1509,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>AQ3</t>
+          <t>EQ3</t>
         </is>
       </c>
       <c r="B4" s="7" t="n">
@@ -1649,7 +1737,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>EQ15</t>
+          <t>CQ15</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
@@ -1761,22 +1849,41 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>CQ15</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E22" s="25" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>AVG</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>5</v>
+      <c r="B23" s="11" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>4.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>